<commit_message>
Feat/added staff testcases (#53)
* Implimentation of "Verify a newly promoted administrator can actually open the admin console"

* Updated Excel sheets

* Updated Dashboard

* updated Dashboard
</commit_message>
<xml_diff>
--- a/testAutomation_v1.0/test/Manual/C1App/AdminApp-Staff/AdminApp_Staff_tab_test_cases.xlsx
+++ b/testAutomation_v1.0/test/Manual/C1App/AdminApp-Staff/AdminApp_Staff_tab_test_cases.xlsx
@@ -102,7 +102,7 @@
     <t>Automated</t>
   </si>
   <si>
-    <t>Suite: adminStaffTab | 2026-09-16: Pass across 2 runs</t>
+    <t>Suite: adminStaffTab | Not executed in this audit - status carried over, treat as unverified</t>
   </si>
   <si>
     <t>TST_STFL_TC_3</t>
@@ -510,7 +510,7 @@
     <t>The row itself is the menu toggle — the whole row is a button with data-toggle="dropdown", and the menu holds exactly ONE item, View profile. There is no "Activate course materials" item as there is on the Students tab. teacher17aug2026@mailsac.com is the team-nominated teacher fixture for this school [confirmed with the team 2026-08-24].</t>
   </si>
   <si>
-    <t>Suite: adminStaffProfile | 2026-09-16: Pass across 2 runs</t>
+    <t>Suite: adminStaffProfile | Not executed in this audit - status carried over, treat as unverified</t>
   </si>
   <si>
     <t>TST_STFP_TC_2</t>
@@ -3325,16 +3325,16 @@
         <v>26</v>
       </c>
       <c r="M40" s="3" t="s">
-        <v>144</v>
+        <v>27</v>
       </c>
       <c r="N40" s="3" t="s">
         <v>26</v>
       </c>
       <c r="O40" s="3" t="s">
-        <v>145</v>
+        <v>28</v>
       </c>
       <c r="P40" s="3" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
     </row>
     <row r="41" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>